<commit_message>
removed RS from rule as this will need more complex programming and record level sensitivity. Will be done in a separate rule.
</commit_message>
<xml_diff>
--- a/rules/CORE-000031/positive/01/data/unit-test-coreid-CG0659-positive.xlsx
+++ b/rules/CORE-000031/positive/01/data/unit-test-coreid-CG0659-positive.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marisa_wyckmans\CORE\CDISC_Rule_Authoring\core-contributor\rules\CORE-000031\positive\01\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\els_janssens\CORE\Rule_Authoring\core-contributor\rules\CORE-000031\positive\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7F7874E-608F-45E3-9D7C-BD08FD3EB636}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6D0DE7B-4DE3-4632-90BC-D5250310A851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21240" windowHeight="15270" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="124">
   <si>
     <t>Product</t>
   </si>
@@ -387,13 +387,22 @@
   </si>
   <si>
     <t>-P2W</t>
+  </si>
+  <si>
+    <t>Evaluator</t>
+  </si>
+  <si>
+    <t>PERSON A</t>
+  </si>
+  <si>
+    <t>RSEVAL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -412,6 +421,15 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -455,7 +473,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -467,6 +485,8 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1177,10 +1197,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="8" max="8" width="9.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>12</v>
       </c>
@@ -1202,38 +1225,41 @@
       <c r="G1" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="90" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" ht="90" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>34</v>
       </c>
@@ -1256,37 +1282,40 @@
         <v>83</v>
       </c>
       <c r="H2" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="I2" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="K2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="L2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="M2" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="O2" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="P2" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="Q2" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="R2" s="3" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>56</v>
       </c>
@@ -1315,17 +1344,17 @@
         <v>56</v>
       </c>
       <c r="J3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="K3" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="K3" s="3" t="s">
-        <v>56</v>
-      </c>
       <c r="L3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="M3" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="M3" s="3" t="s">
-        <v>56</v>
-      </c>
       <c r="N3" s="3" t="s">
         <v>56</v>
       </c>
@@ -1333,13 +1362,16 @@
         <v>56</v>
       </c>
       <c r="P3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q3" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="Q3" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R3" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>12</v>
       </c>
@@ -1362,37 +1394,40 @@
         <v>7</v>
       </c>
       <c r="H4" s="3">
+        <v>200</v>
+      </c>
+      <c r="I4" s="3">
         <v>198</v>
       </c>
-      <c r="I4" s="3">
-        <v>8</v>
-      </c>
       <c r="J4" s="3">
         <v>8</v>
       </c>
       <c r="K4" s="3">
+        <v>8</v>
+      </c>
+      <c r="L4" s="3">
         <v>1</v>
       </c>
-      <c r="L4" s="3">
-        <v>8</v>
-      </c>
       <c r="M4" s="3">
+        <v>8</v>
+      </c>
+      <c r="N4" s="3">
         <v>200</v>
       </c>
-      <c r="N4" s="3">
+      <c r="O4" s="3">
         <v>9</v>
       </c>
-      <c r="O4" s="3">
+      <c r="P4" s="3">
         <v>10</v>
       </c>
-      <c r="P4" s="3">
-        <v>8</v>
-      </c>
       <c r="Q4" s="3">
+        <v>8</v>
+      </c>
+      <c r="R4" s="3">
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="105" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" ht="105" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>58</v>
       </c>
@@ -1414,34 +1449,37 @@
       <c r="G5" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="I5" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="J5" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="J5" s="4">
+      <c r="K5" s="4">
         <v>1</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="L5" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="L5" s="4">
+      <c r="M5" s="4">
         <v>3</v>
       </c>
-      <c r="M5" s="4" t="s">
+      <c r="N5" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="N5" s="4" t="s">
+      <c r="O5" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="O5" s="4" t="s">
+      <c r="P5" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="P5" s="4">
+      <c r="Q5" s="4">
         <v>1</v>
       </c>
-      <c r="Q5" s="4" t="s">
+      <c r="R5" s="4" t="s">
         <v>96</v>
       </c>
     </row>

</xml_diff>